<commit_message>
Normalize actuals month notation to YYYY-MM
工数乖離の主因は「月」列のゼロ埋め有無だった。

案件の月リストは pd.period_range から作られるため常に 'YYYY-MM' だが、
実績側が '2019-4' のようにゼロ埋めされていないと文字列一致せず、
build_project_curves の reindex で丸ごと落ちる。さらに文字列比較では
'2019-4' > '2019-04' となるため、期間内の実績が「契約期間外(終了後)」
として除外され、警告を読んでも真因が桁揃えだと分からなかった。
1〜9月がすべて該当するため被害が大きく、サンプルデータで再現したところ
実績の 74.8% が消失した(修正後は乖離 0.00%)。

_normalize_months() で 2019-4 / 2019/04 / 2019.4 / 201904 / 2019-04-01 /
全角表記などを 'YYYY-MM' に正規化し、表記ゆれを検出した場合と年月として
解釈できない値があった場合をそれぞれ件数・実例つきで警告する。
月の異なり数は高々数百なのでユニーク値だけ変換して貼り直しており、
80万行でも読み込みを含めて 6.4 秒で完走することを確認した。

なお、実績データへの列追加と「時間」の桁揃え(整数/小数3桁の混在)は
集計結果に影響しないことを同じ再現データで確認済み。

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EzcNRY8EVx6HeGCEMZT8ER
</commit_message>
<xml_diff>
--- a/output/forecast_PJ-2026-K_align-on_行程グループ.xlsx
+++ b/output/forecast_PJ-2026-K_align-on_行程グループ.xlsx
@@ -1792,7 +1792,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 12:49</t>
+          <t>2026-09-02 13:03</t>
         </is>
       </c>
     </row>
@@ -11578,7 +11578,7 @@
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>2026-09-02 12:49:38</t>
+          <t>2026-09-02 13:03:48</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Clarify month-notation warning wording
表記が混在している場合にだけ起きる問題だと誤読されうる文言だったので、
実績CSV側の表記が首尾一貫していても発生することを明示する。

ゼロ埋めなしで完全に統一されていても、10〜12月だけが偶然どちらの表記でも
同じ文字列になるため生き残り、1〜9月の9ヶ月分(=約4分の3)が消える。

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EzcNRY8EVx6HeGCEMZT8ER
</commit_message>
<xml_diff>
--- a/output/forecast_PJ-2026-K_align-on_行程グループ.xlsx
+++ b/output/forecast_PJ-2026-K_align-on_行程グループ.xlsx
@@ -1792,7 +1792,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 13:03</t>
+          <t>2026-09-02 13:10</t>
         </is>
       </c>
     </row>
@@ -11578,7 +11578,7 @@
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>2026-09-02 13:03:48</t>
+          <t>2026-09-02 13:10:23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Validate phase_map before it decides what gets aggregated
実績人月は phase_map に載っている行程だけを集計する。その判断材料は
この表だけなので、表が静かに壊れていると実績CSVが正しくても集計対象が
ずれる。検証したところ2つの穴があった。

1. 集約軸の値が空欄の行。groups 一覧に欠損が入り、出力に中身のない列が
   生える。既存の行程名と重複していた場合は、正しく割り当て済みの行程を
   後勝ちで上書きして未マッピングに落とすため、行を足したはずが工数が
   丸ごと除外される(検証では 307 人月)。
2. 実績行程名の重複。マッピングは dict(zip(...)) の後勝ちで、先の割り当てが
   無警告で捨てられる。工数は消えないが別グループに付け替わるので、
   工数比率だけが静かに歪む。

_check_phase_map() を追加し、空欄行は無視したうえで警告、重複は採用される
割り当てを明示して警告するようにした。集約軸は overrides でも変わるため、
settings 確定後に検証している。正常なマスタでは警告ゼロで挙動不変。

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EzcNRY8EVx6HeGCEMZT8ER
</commit_message>
<xml_diff>
--- a/output/forecast_PJ-2026-K_align-on_行程グループ.xlsx
+++ b/output/forecast_PJ-2026-K_align-on_行程グループ.xlsx
@@ -1967,7 +1967,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 14:04</t>
+          <t>2026-09-02 14:14</t>
         </is>
       </c>
     </row>
@@ -38956,7 +38956,7 @@
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>2026-09-02 14:04:01</t>
+          <t>2026-09-02 14:14:26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Learn only from completed projects
学習に使う案件の条件を「ステータス=予測対象 でない」から「ステータス=完了」に
変更した。進行中案件は実績が途中までしか無く、カーブを合計1に正規化してから
平均する都合で「前半にすべて消化する案件」として学習される。

実測(完了30件+進行中5件の実データ想定):
    完了のみ           月次誤差WAPE 0.2716
    進行中も混ぜる      月次誤差WAPE 0.2742  (-1.0%)
完了案件が少ないほど影響が大きく、完了5件のときは 9.1% 悪化した。
途中までの実績を打ち切りとして正しく扱う方式も試したが、完了案件が
十分あれば効果はほぼ無い(同条件で +0.1%)ため、第1版では単純に外す。

除外は他の除外理由と同じくステータス名つきで警告に出す。
ステータスの空欄・前後の空白は「完了」として扱い、想定外の表記は
件数と人月つきで報告するので、取りこぼしても気づける。

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EzcNRY8EVx6HeGCEMZT8ER
</commit_message>
<xml_diff>
--- a/output/forecast_PJ-2026-K_align-on_行程グループ.xlsx
+++ b/output/forecast_PJ-2026-K_align-on_行程グループ.xlsx
@@ -2296,7 +2296,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 22:29</t>
+          <t>2026-09-03 00:32</t>
         </is>
       </c>
     </row>
@@ -16279,7 +16279,7 @@
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>2026-09-02 22:29:47</t>
+          <t>2026-09-03 00:32:33</t>
         </is>
       </c>
     </row>

</xml_diff>